<commit_message>
fix(ux): polish feedback placeholder to dual-mode input, streamline indigenous guides layout & fix relative image paths to root-relative
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/09_IMAGE_ASSETS_HEALTH_AUDIT.xlsx
+++ b/docs/09_IMAGE_ASSETS_HEALTH_AUDIT.xlsx
@@ -433,9 +433,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
@@ -474,7 +474,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>防线核实说明</t>
+          <t>相关性与防线核实说明</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>涵盖锁具门上实景、原厂蓝图、转接件与现场故障照片</t>
+          <t>涵盖真实门上实景、原厂蓝图、12款转接件与现场故障照片</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>70 款锁具 × 3 视角 (210 项引用)</t>
+          <t>72 款锁具 × 3 视角 (216 项引用)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8 款标准转接件与工具</t>
+          <t>12 款标准转接件与工具</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>变径套管、防撬卡爪、万向适配盘与加固垫片实图 100% 匹配</t>
+          <t>变径套管、万向盘、水滴夹具、120mm螺栓与3D悬臂支架实图 100% 匹配</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Markdown 页面内容 (content/pages/)</t>
+          <t>工业索引指南 (indigenous-guides.md)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>全站全部中英 Markdown</t>
+          <t>6 大工业区域核心指南</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0 个失效 (已修复双斜杠)</t>
+          <t>0 个失效 (已全部修复为根相对路径 /assets/)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>已彻底清除 '..//assets/' 历史路径拼写问题</t>
+          <t>德法日澳拉美六大板块原厂刻印与锁体照片完全按物理实物一一对应</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>211 个静态 HTML 页面</t>
+          <t>217 个静态 HTML 页面</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0 个死链 (34项测试断言)</t>
+          <t>0 个死链 (33项测试断言)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
feat(killer-features): assimilate weatherproofing salt-spray, multipoint kinematics, emergency clutch whitelist, and door fastener matrix into all 72 locks
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/09_IMAGE_ASSETS_HEALTH_AUDIT.xlsx
+++ b/docs/09_IMAGE_ASSETS_HEALTH_AUDIT.xlsx
@@ -741,7 +741,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.34 KB</t>
+          <t>2.37 KB</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.36 KB</t>
+          <t>2.39 KB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.29 KB</t>
+          <t>2.33 KB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.04 KB</t>
+          <t>2.07 KB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.05 KB</t>
+          <t>2.08 KB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.84 KB</t>
+          <t>1.87 KB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2.36 KB</t>
+          <t>2.4 KB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.1 KB</t>
+          <t>2.14 KB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.9 KB</t>
+          <t>1.93 KB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.9 KB</t>
+          <t>1.93 KB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.93 KB</t>
+          <t>1.96 KB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.94 KB</t>
+          <t>1.97 KB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2.24 KB</t>
+          <t>2.28 KB</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2.07 KB</t>
+          <t>2.11 KB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2.07 KB</t>
+          <t>2.11 KB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2.07 KB</t>
+          <t>2.1 KB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.32 KB</t>
+          <t>2.35 KB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.32 KB</t>
+          <t>2.35 KB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.32 KB</t>
+          <t>2.36 KB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.45 KB</t>
+          <t>2.49 KB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2.35 KB</t>
+          <t>2.38 KB</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.34 KB</t>
+          <t>2.38 KB</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2.32 KB</t>
+          <t>2.35 KB</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2.32 KB</t>
+          <t>2.35 KB</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2.32 KB</t>
+          <t>2.35 KB</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2.32 KB</t>
+          <t>2.35 KB</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2.14 KB</t>
+          <t>2.17 KB</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2.12 KB</t>
+          <t>2.15 KB</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2.12 KB</t>
+          <t>2.16 KB</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2.11 KB</t>
+          <t>2.14 KB</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">

</xml_diff>